<commit_message>
xlsx file splite into 3 sheets
</commit_message>
<xml_diff>
--- a/output/adorsho poribar-test/book-output.xlsx
+++ b/output/adorsho poribar-test/book-output.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Book Content" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chapter" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="section" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="content" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,15 +439,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="35" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -459,26 +457,6 @@
           <t>chapter_name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>section_id</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>section_name</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>content</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>notes</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -489,15 +467,193 @@
           <t>নারী ও পুরুষের আদর্শ</t>
         </is>
       </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>section_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>section_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>chapter_id</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>নারী ও পুরুষের আদর্শ</t>
+        </is>
+      </c>
       <c r="C2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>নারী ও পুরুষের আদর্শ</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>প্রথম আদর্শ</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>দ্বিতীয় আদর্শ</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>তৃতীয় আদর্শ</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>চতুর্থ আদর্শ</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>পঞ্চম আদর্শ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>ষষ্ঠ আদর্শ</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>content_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>chapter_id</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>section_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;নারী ও পুরুষ উভয়কেই যেমন সৃষ্টিকুলের মধ্যে বিশেষ সম্মানিত করে সৃষ্টি করা হয়েছে, তেমনি ইসলামের দৃষ্টিতে নারী-পুরুষের মধ্যে কিছু বিশেষ গুণের বাস্তবতা কামনা করা হয়েছে। এই গুণগুলোই তাদেরকে আদর্শবান হিসাবে তৈরি করতে পারে এবং একমাত্র এই আদর্শের অধিকারী নারী-পুরুষই ইসলামের দেওয়া মর্যাদা রক্ষা করতে পারে। নারী-পুরুষের পারস্পরিক সম্পর্ক ও তাদের পারিবারিক জীবনের বিবরণ পেশ করার পূর্বে তাদের বিশেষ বিশেষ কিছু গুণাবলি সংক্ষিপ্তভাবে পেশ করা হলো।&lt;/p&gt;
 &lt;p&gt;আল্লাহ তাআলা সূরা আহযাবের ৩৫-৩৬ নং আয়াতে আদর্শ নারী-পুরুষের জন্য ১২টি গুণ পেশ করেছেন। আমরা এইসব গুণাবলির সংক্ষিপ্ত বিবরণ দিয়ে বইয়ের প্রাথমিক আলোচনা আরম্ভ করলাম। আশা করি, নর-নারী সকল পাঠক এসব গুণাবলি অর্জন করে আল্লাহর সন্তুষ্টি লাভে ধন্য হবে। আল্লাহ তুমি কবুল কর-আমীন!&lt;/p&gt;
@@ -506,26 +662,19 @@
 &lt;p&gt;উল্লিখিত আয়াতে আল্লাহ রব্বুল আলামীন এক জন আদর্শ নারী-পুরুষের জন্য এমন কিছু গুণাবলি বা বৈশিষ্ট্যের কথা উল্লেখ করেছেন। সেই গুণাবলি যদি কোন নারী-পুরুষের মাঝে বিদ্যমান থাকে, তাহলে তার জন্য মহাপুরস্কারের ঘোষণা দিয়েছেন। উল্লিখিত আয়াতে নারী-পুরুষের জন্য ১২টি শিক্ষণীয়, গ্রহণীয় ও অবশ্য পালনীয় আদর্শ রয়েছে। যা ধারাবাহিকভাবে উল্লেখ করা হলো।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>নারী ও পুরুষের আদর্শ</t>
-        </is>
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>প্রথম আদর্শ</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;মুসলিম পুরুষ ও মুসলিম স্ত্রীলোক। 'মুসলিম' শব্দের আভিধানিক অর্থ আত্মসমর্পণকারী। আর পারিভাষিক অর্থে আল্লাহ ও তাঁর রাসূল (ﷺ)-এর আঈন পালনকারী। আর পারিভাষিক অর্থ হচ্ছে, সুস্থতায়, অসুস্থতায়, সুখে, দুঃখে, সর্বময় ক্ষমতাধর আল্লাহ তাআলার নিকটে নতশীরে ইসলামের যাবতীয় বিধি-বিধান মেনে নেওয়া।&lt;/p&gt;
 &lt;p&gt;এক জন আদর্শ মানুষ হওয়ার জন্য বা প্রকৃত মুসলিম হওয়ার জন্য রাসূলুল্লাহ (ﷺ) কিছু গুণাবলির কথা উল্লেখ করেছেন। যেমন রাসূলুল্লাহ (ﷺ)-এর বাণী-&lt;/p&gt;
@@ -543,26 +692,19 @@
 &lt;p&gt;উপরিউক্ত আলোচনায় একজন মুসলিমের যে বৈশিষ্ট্য গুলো থাকা জরুরী তা নিচে আলোচনা করা হলো।&lt;br&gt;১. ইসলামে প্রবেশ করার জন্য প্রথমেই আল্লাহ তাআলার প্রতি বিশ্বাস স্থাপন করা। মুহাম্মাদ (ﷺ)-কে তাঁর রাসূল বা নবী হিসাবে বিশ্বাস করা।&lt;br&gt;২. দিনে-রাতে পাঁচ ওয়াক্ত ছালাত আদায় করা।&lt;br&gt;৩. নিসাব পরিমান সম্পদ থাকলে যাকাত প্রদান করা।&lt;br&gt;৪. রমাযান মাসে ছিয়াম পালন করা।&lt;br&gt;৫. সামর্থ্য থাকলে হজ্জ করা।&lt;br&gt;৬. অপর মুসলিমকে কষ্ট না দেওয়া।&lt;br&gt;৭. আত্মীয়তার সম্পর্ক ছিন্ন না করা।&lt;br&gt;৮. কোনো মুসলিম ভাই রোগাক্রান্ত হলে তাকে দেখতে যাওয়া এবং তার সেবা-শুশ্রুষা করা।&lt;br&gt;৯. কোন মুসলিম মারা গেলে তার জানাযায় উপস্থিত থাকা।&lt;br&gt;১০. কোন মুসলিম দাওয়াত করলে তার দাওয়াতে সাড়া দেওয়া।&lt;br&gt;১১. পরস্পর সকল মুসলিমকে সাক্ষাতকালে সালাম দেওয়া। আমাদের দেশে সামাজিক একটি কুঅভ্যাস চালু হয়েছে তাহল, শুধু পরিচিত সম্মানীদেরকে সালাম দেয়। আর যারা সম্মানী তারাও মনে করে যে, আমাদেরকে সালাম দিক যা সম্পূর্ণ হারাম। এটাই অনুসরণীয় যে, পরিচিত-অপরিচিত, ছোট-বড় সকলকে সালাম দিতে হবে। কেননা ঐ ব্যক্তি সর্ব উত্তম, যে আগে সালাম দেয়।&lt;br&gt;১২. কোন মুসলিম হাঁচি দিলে তার উত্তরে 'ইয়ারহামুকা-ল্লাহ' বলা, আর হাঁচি দাতার 'ইয়াহদীকুমু-ল্লাহ' বলা।&lt;br&gt;১৩. সর্ব অবস্থায় এক জন মুসলিম অপর মুসলিমের জন্য কল্যাণ কামনা করা এবং সুপরামর্শ দেওয়া। উপরোক্ত গুনাবলি যদি কারো মধ্যে না থাকে, তাহলে সে পূর্ণ মুসলিম নয় অতএব উপরিউক্ত গুণাবলি এক জন মুসলিমের মধ্যে থাকা জরুরী।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>নারী ও পুরুষের আদর্শ</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>দ্বিতীয় আদর্শ</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;মু'মিন পুরুষ ও মু'মিন নারী। 'মু'মিন' শব্দের অর্থ হচ্ছে, ঈমানদার। পরিভাষায় ঈমান হচ্ছে, একনিষ্ঠভাবে আল্লাহকে একমাত্র উপাস্য হিসেবে বিশ্বাস করা, রাসূলগণকে আল্লাহ তাআলার প্রেরিত রাসূল হিসেবে বিশ্বাস করা, পবিত্র কোরআন ও পূর্ববর্তী কিতাবসমূহের প্রতি বিশ্বাস করা, ফেরেশতাগণের প্রতি বিশ্বাস করা, কিয়ামত দিবসের প্রতি বিশ্বাস করা, তাক্বদীরের ভাল-মন্দের প্রতি বিশ্বাস স্থাপন করা, যেমন আল্লাহ তাআলার বাণী,&lt;/p&gt;
 &lt;ar&gt;آمَنَ الرَّسُولُ بِمَا أُنْزِلَ إِلَيْهِ مِنْ رَبِّهِ وَالْمُؤْمِنُونَ كُلٌّ آمَنَ بِاللَّهِ وَمَلَا بِكَتِهِ وَكُتُبِهِ وَرُسُلِهِ لَا نُفَرِّقُ بَيْنَ أَحَدٍ مِنْ رُسُلِهِ وَقَالُوا سَمِعْنَا وَأَطَعْنَا غُفْرَانَكَ رَبَّنَا وَإِلَيْكَ الْمَصِيرُ।&lt;/ar&gt;
@@ -625,26 +767,19 @@
 &lt;p&gt;'মু'মিন তো তারাই, যাঁদের সামনে আল্লাহ তাআলার কথা স্মরণ করা হলে, তাদের অন্তর কেঁপে ওঠে। আর যখন তাঁদের সামনে আল্লাহ তাআলার আয়াত পাঠ করা হয়, তখন তা তাঁদের ঈমানকে বৃদ্ধি করে। তাঁরা ছালাত কায়েম করে এবং আমার দেওয়া রিযিক্ক হতে দান করে। এরাই হলো প্রকৃত মু'মিন, যাঁদের জন্য তাঁদের প্রতিপালকের নিকটে রয়েছে অগণিত মর্যাদা, ক্ষমা ও সম্মানজনক রিযিকের ব্যবস্থা' (আল-আনফাল, ১-৪)।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>নারী ও পুরুষের আদর্শ</t>
-        </is>
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>তৃতীয় আদর্শ</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;আল্লাহর দিকে মনোনিবেশকারী পুরুষ ও স্ত্রীলোক। এমন পুরুষ ও স্ত্রীলোকের কথা আল্লাহ এখানে বলেছেন, যাদের অন্তর ও দেহের সকল অঙ্গ-প্রত্যঙ্গ সর্বদা আল্লাহর বিধান পালনে মশগুল।&lt;/p&gt;
 &lt;p&gt;আল্লাহ তাআলা বলেন,&lt;/p&gt;
@@ -677,26 +812,19 @@
 &lt;p&gt;উপরিউক্ত আলোচনা হতে এটাই প্রতীয়মান হয় যে, আদর্শ নারী-পুরুষ হিসাবে একমাত্র একনিষ্ঠ ভাবে আল্লাহর ইবাদত করা (শুকুর-গুজার, তাসবীহ-তাহলীল পাঠ করা)।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>নারী ও পুরুষের আদর্শ</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>চতুর্থ আদর্শ</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;সত্য ও ন্যায়-নিষ্ঠ পুরুষ ও স্ত্রীলোক। সততা নারী-পুরুষের জন্য একটি প্রশংসনীয় আদর্শ। সততা এমন ঈমানের পরিচায়ক যার পরিণাম জান্নাত। সত্য যে একটি মহৎ গুণ এবং তার পরিণাম যে জান্নাত, সে ব্যাপারে মহান আল্লাহ বলেন,&lt;/p&gt;
 &lt;ar&gt;وَالْعَصْرِ إِنَّ الْإِنْسَانَ لَفِي خُسْرٍ إِلَّا الَّذِينَ آمَنُوا وَعَمِلُوا الصَّالِحَاتِ وَتَوَاصَوْا بِالْحَقِّ وَتَوَاصَوْا بِالصَّبْرِ.&lt;/ar&gt;
@@ -718,26 +846,19 @@
 &lt;p&gt;কা'ব (রাঃ) বলেন, 'এ শব্দ আমার কানে পৌঁছামাত্র আমি সিজদায় পড়ে গেলাম। আর আমি বুঝলাম যে, আমার সুদিন ও খুশির খবর এসেছে'। আমি আরয করলাম, হে আল্লাহর রাসূল! আল্লাহ তাআলা সত্য কথা বলার কারণে আমাকে রক্ষা করেছেন, তাই আমার তওবা কবুলের নিদর্শন ঠিক রাখতে, আমার বাকী জীবনে সত্য কথাই বলব। আল্লাহর কসম! যখন থেকে আমি এ সত্য বলার কথা রাসূলুল্লাহ (ﷺ)-এর কাছে জানিয়েছি, তখন থেকে আজ পর্যন্ত আমার জানা মতে কোন মুসলিমকে সত্য কথার বিনিময়ে এরূপ নিয়ামত আল্লাহ দান করেননি, যে নিয়ামত আমাকে দান করেছেন।&lt;/p&gt;&lt;br&gt;&lt;br&gt;&lt;p&gt;কা'ব (রাঃ) বলেন, 'যে দিন রাসূলুল্লাহ (ﷺ)-এর সম্মুখে সত্য কথা বলেছি, সেদিন হতে আজ পর্যন্ত অন্তরে মিথ্যা বলার ইচ্ছাও করিনি। আমি আশা পোষণ করি যে, বাকী জীবনও আল্লাহ তাআলা আমাকে মিথ্যা থেকে রক্ষা করবেন' (ছহীহ বুখারী, হা/৪৪১৮)। উপরিউক্ত আলোচনা হতে প্রতীয়মান হয় যে, সত্য ও সততা মানব জীবনে একটি মহৎ গুণ। সত্য ও সততার কারণে সাময়িকভাবে পৃথিবী সংকুচিত হলেও তার ফলাফল অনেক অনেকগুণে সাফল্যজনক ও মর্যাদাপূর্ণ হয়।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>নারী ও পুরুষের আদর্শ</t>
-        </is>
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>পঞ্চম আদর্শ</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;ছবরকারী বা সত্যের পথে দৃঢ়তা প্রদর্শনকারী পুরুষ ও স্ত্রীলোক। 'ছবর'- এর আভিধানিক অর্থ হচ্ছে, নিজেকে বেঁধে রাখা, ধৈর্য ধারণ করা। এখানে এমন পুরুষ ও নারীকে বোঝানো হয়েছে, যারা বিপদে-আপদে আল্লাহর দ্বীন পালন ও তাঁর ইবাদত করতে গিয়ে সকল প্রকার দুঃখ কষ্ট অকাতরে সহ্য করে অটল হয়ে থাকে। শত বাঁধার মোক্কাবিলা করে দ্বীনের উপর অবিচল থাকে এবং কোনক্রমেই আদর্শচ্যুত হয় না। আল্লাহ তাআলা বলেন,&lt;/p&gt;
 &lt;ar&gt;سَلامٌ عَلَيْكُمْ بِمَا صَبَرْتُمْ فَنِعْمَ عُقْبَى الدَّارِ.&lt;/ar&gt;
@@ -819,26 +940,19 @@
 &lt;p&gt;উপরিউক্ত আলোচনা হতে এটাই প্রতীয়মান হয় যে, সুখে-দুঃখে, বালা, মছিবতে রোগ-যন্ত্রণায়, অত্যাচারীদের অত্যাচারে সর্বাবস্থায় ধৈর্যধারণ করাই প্রকৃত মু'মিনের কাজ। আর পরস্পরকে ধৈর্যধারণের উপদেশ দিতে হবে এবং নিজেদেরকেও ধৈর্যধারণ করতে হবে।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>নারী ও পুরুষের আদর্শ</t>
-        </is>
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="C8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>ষষ্ঠ আদর্শ</t>
-        </is>
-      </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>&lt;div class="page-text"&gt;&lt;p&gt;আল্লাহর নিকট বিনীত-নম্র পুরুষ ও স্ত্রীলোক। আল্লাহ তাআলা এখানে এমন নারী-পুরুষের আদর্শ বর্ণনা করেছেন, যারা অন্তর-মন ও অঙ্গ-প্রত্যঙ্গ সব কিছু দিয়ে বিনীতভাবে আল্লাহ তাআলার ইবাদত করে। এখানে এমন এক শব্দ উল্লিখিত হয়েছে যার অর্থ- প্রশান্তি, স্থিতি, প্রীতি, শ্রদ্ধা, ভক্তি, বিনয়, ভয় মিশ্রিত ভালোবাসা এবং আল্লাহ তাআলার প্রতি আগ্রহ, উৎসাহ। আল্লাহ তাআলা বলেন,&lt;/p&gt;
 &lt;ar&gt;قَدْ أَفْلَحَ الْمُؤْمِنُونَ الَّذِينَ هُمْ فِي صَلَاتِهِمْ خَاشِعُونَ.&lt;/ar&gt;
@@ -873,7 +987,7 @@
 &lt;p&gt;উপর্যুক্ত হাদীছ দ্বারা বুঝা যায় যে, পাঁচ ওয়াক্ত ফরজ ছালাত আদায়ের পরেও আল্লাহ তাআলার ভয়ে বিনীতভাবে রাত্রি জাগরণ করে নফল ছালাত আদায় করা, আদর্শ নারী-পুরুষের কাজ।&lt;/p&gt;&lt;/div&gt;</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>